<commit_message>
docs: 집구경(TOUR-01/02) PC 지원 정합 (화면설계서 v8.0)
PC 집구경 Figma 노드(135:2921 갤러리·135:3135 라이트박스) 확인·구현 반영.
- 화면설계서: TOUR-01/02 PC ✕→O, node-id 추가, 설명에 의도적 편차 주석(Figma 갱신 예정), 변경이력 v8.0
- design_nodeId.md: PC 집구경 노드 추가

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ZIPBODA_화면설계서_v0.1.xlsx
+++ b/docs/ZIPBODA_화면설계서_v0.1.xlsx
@@ -683,10 +683,24 @@
       <c r="F8" s="7" t="n"/>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="20">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>사용자용</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>집구경(TOUR-01/02) PC 지원 반영 — Figma PC 노드(135:2921 갤러리·135:3135 라이트박스) 확인·구현, PC ✕→O·node-id 추가. 구현이 Figma PC 대비 의도적 개선분 있어 편차 기록(Figma 갱신 예정).</t>
+        </is>
+      </c>
       <c r="E9" s="7" t="n"/>
       <c r="F9" s="7" t="n"/>
     </row>
@@ -9697,7 +9711,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>(공통) '인테리어 영감' 갤러리. 공간 카테고리(전체/거실/침실/주방/다이닝/서재/욕실) 탭 + 실제 유저 홈 사진 그리드(@핸들·❤️ 좋아요).</t>
+          <t>(공통) '인테리어 영감' 갤러리. 공간 카테고리(전체/거실/침실/주방/다이닝/서재/욕실) 탭 + 실제 유저 홈 사진 그리드(@핸들·❤️ 좋아요). (PC 지원 반영 — 갤러리. 구현이 Figma PC와 일부 상이한 의도적 개선분 있음, Figma 갱신 예정)</t>
         </is>
       </c>
       <c r="G13" s="17" t="inlineStr">
@@ -9747,7 +9761,7 @@
       </c>
       <c r="P13" s="0" t="inlineStr">
         <is>
-          <t>✕</t>
+          <t>O</t>
         </is>
       </c>
       <c r="Q13" s="0" t="inlineStr">
@@ -9757,7 +9771,7 @@
       </c>
       <c r="R13" s="0" t="inlineStr">
         <is>
-          <t>— / 1:1851</t>
+          <t>135:2921 / 1:1851</t>
         </is>
       </c>
     </row>
@@ -9787,7 +9801,7 @@
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>(공통) 인테리어 사진 상세(작성자·좋아요)와 '이 스타일 쇼핑하기'로 사진 속 가구 쇼핑 유도.</t>
+          <t>(공통) 인테리어 사진 상세(작성자·좋아요)와 '이 스타일 쇼핑하기'로 사진 속 가구 쇼핑 유도. (PC는 갤러리 내 라이트박스로 구현. Figma PC 대비 개선분 있음, Figma 갱신 예정)</t>
         </is>
       </c>
       <c r="G14" s="17" t="inlineStr">
@@ -9837,7 +9851,7 @@
       </c>
       <c r="P14" s="0" t="inlineStr">
         <is>
-          <t>✕</t>
+          <t>O</t>
         </is>
       </c>
       <c r="Q14" s="0" t="inlineStr">
@@ -9847,7 +9861,7 @@
       </c>
       <c r="R14" s="0" t="inlineStr">
         <is>
-          <t>— / 1:1976</t>
+          <t>135:3135 / 1:1976</t>
         </is>
       </c>
     </row>

</xml_diff>